<commit_message>
Complete Signup functional testing: test cases, bug reports BUG-002 to BUG-004, and evidence
</commit_message>
<xml_diff>
--- a/Test Cases/Signup_Test_Cases.xlsx
+++ b/Test Cases/Signup_Test_Cases.xlsx
@@ -329,7 +329,7 @@
     <t>Form gönderilmedi, ancak gösterilen hata mesajı ("Şifre, geçersiz karakterler içermemelidir.") yanıltıcıydı — asıl sorun büyük harf eksikliğiydi, geçersiz karakter değil. Aynı genel mesaj, farklı şifre kuralı ihlallerinde (kısa uzunluk, büyük harf eksikliği) tekrar tekrar çıktı, gerçek kuralı yansıtmıyor.</t>
   </si>
   <si>
-    <t>Evidence/Screenshots/TC-SIGNUP-006_misleading_password_error.png</t>
+    <t xml:space="preserve">Evidence/Screenshots/TC-SIGNUP-006_misleading_password_error.png  ,See Bug Reports/BUG-002.pdf</t>
   </si>
   <si>
     <t>FAIL</t>
@@ -376,7 +376,7 @@
     <t>Form gönderilmedi, ancak yine aynı genel/yanıltıcı hata mesajı ("Şifre, geçersiz karakterler içermemelidir.") çıktı, eksik rakam kuralına özgü bir mesaj değil. Şifre gücü göstergesi de güncellenmedi.</t>
   </si>
   <si>
-    <t>Evidence/Screenshots/TC-SIGNUP-007_misleading_password_error.png</t>
+    <t>Evidence/Screenshots/TC-SIGNUP-007_misleading_password_error.png ,See Bug Reports/BUG-002.pdf</t>
   </si>
   <si>
     <t>TC-SIGNUP-008</t>
@@ -420,7 +420,7 @@
     <t>Form gönderilmedi, ancak yine aynı genel/yanıltıcı hata mesajı çıktı, eksik özel karakter kuralına özgü değil. Şifre gücü göstergesi güncellenmedi, kural listesi de özel karakter kuralı karşılanmamışken 4 kuralın da karşılandığını gösterdi.</t>
   </si>
   <si>
-    <t>Evidence/Screenshots/TC-SIGNUP-008_misleading_password_error.png</t>
+    <t>Evidence/Screenshots/TC-SIGNUP-008_misleading_password_error.png ,See Bug Reports/BUG-002.pdf</t>
   </si>
   <si>
     <t>TC-SIGNUP-009</t>
@@ -462,7 +462,7 @@
     <t>Hesap başarıyla oluşturuldu ve kullanıcı Giriş sayfasına yönlendirildi. Ancak şifre tüm 4 kuralı karşılamasına rağmen, gösterge hiçbir seviye göstermedi (boş kaldı), beklenen "Strong/Very Strong/Excellent" davranışıyla çelişti.</t>
   </si>
   <si>
-    <t>Evidence/Screenshots/TC-SIGNUP-009_strength_indicator_blank.png</t>
+    <t>Evidence/Screenshots/TC-SIGNUP-009_strength_indicator_blank.png ,See Bug Reports/BUG-003.pdf</t>
   </si>
   <si>
     <t>Low</t>
@@ -509,7 +509,7 @@
     <t>Sokak alanı doğru şekilde otomatik doldu. Ancak Şehir alanı, 35000 posta koduna (İzmir'e ait) uymayan yanlış bir değerle ("Elazığ") dolduruldu, Eyalet alanı ise hiç otomatik dolmadı — boş kaldı ve elle girilmesi gerekti.</t>
   </si>
   <si>
-    <t>Evidence/Screenshots/TC-SIGNUP-010_autofill_city_state_bug.png</t>
+    <t>Evidence/Screenshots/TC-SIGNUP-010_autofill_city_state_bug.png ,See Bug Reports/BUG-004.pdf</t>
   </si>
   <si>
     <t>TC-SIGNUP-011</t>

</xml_diff>